<commit_message>
Merged PR 2215: Merge MahadevProductB to master
projectManager.java - added a new method for flex table quick search
and fixed scenarios in site visit and desk review
</commit_message>
<xml_diff>
--- a/src/main/resources/DeskReview_Field_Values.xlsx
+++ b/src/main/resources/DeskReview_Field_Values.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="21328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="21601"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\govgrants-product-automation\src\main\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Workspace-Product-Automation\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A5E4A85-CEB9-4C47-9968-183639FAAE8A}" xr6:coauthVersionLast="41" xr6:coauthVersionMax="41" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA2B53C0-3A1F-44C1-A569-0D9517B27096}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="3" xr2:uid="{9AB3C168-78A6-4CA6-B0EE-C4F246080D71}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{9AB3C168-78A6-4CA6-B0EE-C4F246080D71}"/>
   </bookViews>
   <sheets>
     <sheet name="Creation" sheetId="1" r:id="rId1"/>
@@ -83,36 +83,21 @@
     <t>VisitEndDateTime__c</t>
   </si>
   <si>
-    <t>Description__c</t>
-  </si>
-  <si>
     <t>RichText</t>
   </si>
   <si>
     <t>Automation Test description</t>
   </si>
   <si>
-    <t>Pointsdiscussedwithofficials__c</t>
-  </si>
-  <si>
-    <t>SiteVisitPurpose__c</t>
-  </si>
-  <si>
     <t>Dropdown</t>
   </si>
   <si>
     <t>Routine based on monitoring responsibilities</t>
   </si>
   <si>
-    <t>SourceSiteVisit__c</t>
-  </si>
-  <si>
     <t>To fulfill pass-through monitoring responsibilities</t>
   </si>
   <si>
-    <t>SupportingCommentsQuestion1__c</t>
-  </si>
-  <si>
     <t>TextArea</t>
   </si>
   <si>
@@ -354,13 +339,28 @@
   </si>
   <si>
     <t>2. If hiring is to occur, does the agency adhere to Federal and State EEOC (Equal employment Opportunity Act) policies and procedures?</t>
+  </si>
+  <si>
+    <t>fieldDescription__c</t>
+  </si>
+  <si>
+    <t>fieldPointsdiscussedwithofficials__c</t>
+  </si>
+  <si>
+    <t>fieldSiteVisitPurpose__c</t>
+  </si>
+  <si>
+    <t>fieldSourceSiteVisit__c</t>
+  </si>
+  <si>
+    <t>fieldSupportingCommentsQuestion1__c</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -369,12 +369,7 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="8"/>
-      <color rgb="FF6D6D6D"/>
-      <name val="Helvetica"/>
-    </font>
-    <font>
-      <sz val="7"/>
+      <sz val="9"/>
       <color rgb="FF222222"/>
       <name val="Consolas"/>
       <family val="3"/>
@@ -400,7 +395,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -409,7 +404,6 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -725,13 +719,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27F20A35-8E6F-4015-873C-76781E4C62A4}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="20.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="31.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="31.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -742,7 +736,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -750,10 +744,10 @@
         <v>6</v>
       </c>
       <c r="C2" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -764,7 +758,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>4</v>
       </c>
@@ -783,14 +777,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4969FD67-2E2F-4920-8A24-9B3F6A7CB976}">
   <dimension ref="A1:C8"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="8.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.21875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="41.21875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="41.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -801,7 +795,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>13</v>
       </c>
@@ -812,7 +806,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>13</v>
       </c>
@@ -823,76 +817,77 @@
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>13</v>
       </c>
-      <c r="B4" t="s">
-        <v>17</v>
+      <c r="B4" s="3" t="s">
+        <v>103</v>
       </c>
       <c r="C4" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>13</v>
       </c>
-      <c r="B5" t="s">
-        <v>20</v>
+      <c r="B5" s="3" t="s">
+        <v>104</v>
       </c>
       <c r="C5" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>13</v>
       </c>
-      <c r="B6" t="s">
-        <v>21</v>
+      <c r="B6" s="3" t="s">
+        <v>105</v>
       </c>
       <c r="C6" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>13</v>
       </c>
-      <c r="B7" t="s">
-        <v>24</v>
+      <c r="B7" s="3" t="s">
+        <v>106</v>
       </c>
       <c r="C7" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>13</v>
       </c>
-      <c r="B8" t="s">
-        <v>26</v>
+      <c r="B8" s="3" t="s">
+        <v>107</v>
       </c>
       <c r="C8" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{08D4F942-EBC7-4392-9497-9CD173C449CD}">
   <dimension ref="A1:C30"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="21.88671875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="106.21875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="106.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -903,323 +898,323 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>4</v>
       </c>
       <c r="B2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C2" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C3" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4" t="s">
+        <v>27</v>
+      </c>
+      <c r="C4" t="s">
         <v>28</v>
       </c>
-      <c r="C2" t="s">
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>4</v>
-      </c>
-      <c r="B3" t="s">
+      <c r="C5" t="s">
         <v>30</v>
       </c>
-      <c r="C3" t="s">
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>4</v>
+      </c>
+      <c r="B6" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>4</v>
-      </c>
-      <c r="B4" t="s">
+      <c r="C6" t="s">
         <v>32</v>
       </c>
-      <c r="C4" t="s">
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>4</v>
+      </c>
+      <c r="B7" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>4</v>
-      </c>
-      <c r="B5" t="s">
+      <c r="C7" t="s">
         <v>34</v>
       </c>
-      <c r="C5" t="s">
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>4</v>
+      </c>
+      <c r="B8" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>4</v>
-      </c>
-      <c r="B6" t="s">
+      <c r="C8" t="s">
         <v>36</v>
       </c>
-      <c r="C6" t="s">
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>4</v>
+      </c>
+      <c r="B9" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>4</v>
-      </c>
-      <c r="B7" t="s">
+      <c r="C9" t="s">
         <v>38</v>
       </c>
-      <c r="C7" t="s">
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>4</v>
+      </c>
+      <c r="B10" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>4</v>
-      </c>
-      <c r="B8" t="s">
+      <c r="C10" t="s">
         <v>40</v>
       </c>
-      <c r="C8" t="s">
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>4</v>
+      </c>
+      <c r="B11" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>4</v>
-      </c>
-      <c r="B9" t="s">
+      <c r="C11" t="s">
         <v>42</v>
       </c>
-      <c r="C9" t="s">
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>4</v>
+      </c>
+      <c r="B12" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
-        <v>4</v>
-      </c>
-      <c r="B10" t="s">
+      <c r="C12" t="s">
         <v>44</v>
       </c>
-      <c r="C10" t="s">
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>4</v>
+      </c>
+      <c r="B13" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
-        <v>4</v>
-      </c>
-      <c r="B11" t="s">
+      <c r="C13" t="s">
         <v>46</v>
       </c>
-      <c r="C11" t="s">
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>4</v>
+      </c>
+      <c r="B14" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
-        <v>4</v>
-      </c>
-      <c r="B12" t="s">
+      <c r="C14" t="s">
         <v>48</v>
       </c>
-      <c r="C12" t="s">
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>4</v>
+      </c>
+      <c r="B15" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A13" t="s">
-        <v>4</v>
-      </c>
-      <c r="B13" t="s">
+      <c r="C15" t="s">
         <v>50</v>
       </c>
-      <c r="C13" t="s">
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>4</v>
+      </c>
+      <c r="B16" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A14" t="s">
-        <v>4</v>
-      </c>
-      <c r="B14" t="s">
+      <c r="C16" t="s">
         <v>52</v>
       </c>
-      <c r="C14" t="s">
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>4</v>
+      </c>
+      <c r="B17" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A15" t="s">
-        <v>4</v>
-      </c>
-      <c r="B15" t="s">
+      <c r="C17" t="s">
         <v>54</v>
       </c>
-      <c r="C15" t="s">
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>4</v>
+      </c>
+      <c r="B18" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A16" t="s">
-        <v>4</v>
-      </c>
-      <c r="B16" t="s">
+      <c r="C18" t="s">
         <v>56</v>
       </c>
-      <c r="C16" t="s">
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>4</v>
+      </c>
+      <c r="B19" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A17" t="s">
-        <v>4</v>
-      </c>
-      <c r="B17" t="s">
+      <c r="C19" t="s">
         <v>58</v>
       </c>
-      <c r="C17" t="s">
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>4</v>
+      </c>
+      <c r="B20" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A18" t="s">
-        <v>4</v>
-      </c>
-      <c r="B18" t="s">
+      <c r="C20" t="s">
         <v>60</v>
       </c>
-      <c r="C18" t="s">
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>4</v>
+      </c>
+      <c r="B21" t="s">
         <v>61</v>
       </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A19" t="s">
-        <v>4</v>
-      </c>
-      <c r="B19" t="s">
+      <c r="C21" t="s">
         <v>62</v>
       </c>
-      <c r="C19" t="s">
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>4</v>
+      </c>
+      <c r="B22" t="s">
         <v>63</v>
       </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A20" t="s">
-        <v>4</v>
-      </c>
-      <c r="B20" t="s">
+      <c r="C22" t="s">
         <v>64</v>
       </c>
-      <c r="C20" t="s">
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>4</v>
+      </c>
+      <c r="B23" t="s">
         <v>65</v>
       </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A21" t="s">
-        <v>4</v>
-      </c>
-      <c r="B21" t="s">
+      <c r="C23" t="s">
         <v>66</v>
       </c>
-      <c r="C21" t="s">
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>4</v>
+      </c>
+      <c r="B24" t="s">
         <v>67</v>
       </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A22" t="s">
-        <v>4</v>
-      </c>
-      <c r="B22" t="s">
+      <c r="C24" t="s">
         <v>68</v>
       </c>
-      <c r="C22" t="s">
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>4</v>
+      </c>
+      <c r="B25" t="s">
         <v>69</v>
       </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A23" t="s">
-        <v>4</v>
-      </c>
-      <c r="B23" t="s">
+      <c r="C25" t="s">
         <v>70</v>
       </c>
-      <c r="C23" t="s">
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>4</v>
+      </c>
+      <c r="B26" t="s">
         <v>71</v>
       </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A24" t="s">
-        <v>4</v>
-      </c>
-      <c r="B24" t="s">
+      <c r="C26" t="s">
         <v>72</v>
       </c>
-      <c r="C24" t="s">
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>4</v>
+      </c>
+      <c r="B27" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A25" t="s">
-        <v>4</v>
-      </c>
-      <c r="B25" t="s">
+      <c r="C27" t="s">
         <v>74</v>
       </c>
-      <c r="C25" t="s">
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>4</v>
+      </c>
+      <c r="B28" t="s">
         <v>75</v>
       </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A26" t="s">
-        <v>4</v>
-      </c>
-      <c r="B26" t="s">
+      <c r="C28" t="s">
         <v>76</v>
       </c>
-      <c r="C26" t="s">
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>4</v>
+      </c>
+      <c r="B29" t="s">
         <v>77</v>
       </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A27" t="s">
-        <v>4</v>
-      </c>
-      <c r="B27" t="s">
+      <c r="C29" t="s">
         <v>78</v>
       </c>
-      <c r="C27" t="s">
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>4</v>
+      </c>
+      <c r="B30" t="s">
         <v>79</v>
       </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A28" t="s">
-        <v>4</v>
-      </c>
-      <c r="B28" t="s">
-        <v>80</v>
-      </c>
-      <c r="C28" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A29" t="s">
-        <v>4</v>
-      </c>
-      <c r="B29" t="s">
-        <v>82</v>
-      </c>
-      <c r="C29" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A30" t="s">
-        <v>4</v>
-      </c>
-      <c r="B30" t="s">
-        <v>84</v>
-      </c>
       <c r="C30" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
     </row>
   </sheetData>
@@ -1230,14 +1225,14 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1EEE61CD-3237-422A-82E8-CA9710108D17}">
   <dimension ref="A1:C10"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.88671875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="91.21875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="91.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1248,103 +1243,103 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="B2" s="4" t="s">
-        <v>76</v>
-      </c>
-      <c r="C2" s="3" t="s">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" t="s">
+        <v>71</v>
+      </c>
+      <c r="C2" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" t="s">
+        <v>73</v>
+      </c>
+      <c r="C3" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4" t="s">
+        <v>75</v>
+      </c>
+      <c r="C4" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>77</v>
+      </c>
+      <c r="C5" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>4</v>
+      </c>
+      <c r="B6" t="s">
+        <v>89</v>
+      </c>
+      <c r="C6" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>4</v>
+      </c>
+      <c r="B7" t="s">
+        <v>90</v>
+      </c>
+      <c r="C7" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="C3" s="3" t="s">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>4</v>
+      </c>
+      <c r="B8" t="s">
+        <v>91</v>
+      </c>
+      <c r="C8" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>80</v>
-      </c>
-      <c r="C4" s="3" t="s">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>4</v>
+      </c>
+      <c r="B9" t="s">
+        <v>92</v>
+      </c>
+      <c r="C9" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>82</v>
-      </c>
-      <c r="C5" s="3" t="s">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>4</v>
+      </c>
+      <c r="B10" t="s">
+        <v>93</v>
+      </c>
+      <c r="C10" t="s">
         <v>102</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>94</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>95</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A8" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>96</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A9" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="B9" s="4" t="s">
-        <v>97</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A10" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="B10" s="4" t="s">
-        <v>98</v>
-      </c>
-      <c r="C10" s="3" t="s">
-        <v>107</v>
       </c>
     </row>
   </sheetData>
@@ -1356,12 +1351,12 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BFC7A54C-E16D-458B-92CE-DB4DE5E21708}">
   <dimension ref="A1:B8"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="9.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -1369,7 +1364,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -1377,7 +1372,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>7</v>
       </c>
@@ -1385,32 +1380,32 @@
         <v>14</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>10</v>
       </c>
       <c r="B4" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B7" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B8" t="s">
         <v>22</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="B7" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="B8" t="s">
-        <v>27</v>
       </c>
     </row>
   </sheetData>
@@ -1421,14 +1416,14 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7B6B17DB-D82F-41EF-9E76-B6B556CE0B3E}">
   <dimension ref="A1:C5"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="19.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="20.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1439,48 +1434,48 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>6</v>
       </c>
       <c r="C2" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="C3" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="B4" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="C4" t="s">
         <v>87</v>
       </c>
-      <c r="C4" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="B5" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="C5" t="s">
         <v>88</v>
-      </c>
-      <c r="C5" t="s">
-        <v>93</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Merged PR 2665: Merge Deepika_prod to master
Created and Automated 10 New Test Cases in Site Visit/Desk Review Features
</commit_message>
<xml_diff>
--- a/src/main/resources/DeskReview_Field_Values.xlsx
+++ b/src/main/resources/DeskReview_Field_Values.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="21601"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="21727"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Workspace-Product-Automation\govgrants-product-automation\src\main\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA2B53C0-3A1F-44C1-A569-0D9517B27096}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{027C3F22-D88C-4FD7-AD12-3CAD3626E955}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{9AB3C168-78A6-4CA6-B0EE-C4F246080D71}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{9AB3C168-78A6-4CA6-B0EE-C4F246080D71}"/>
   </bookViews>
   <sheets>
     <sheet name="Creation" sheetId="1" r:id="rId1"/>
@@ -719,13 +719,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27F20A35-8E6F-4015-873C-76781E4C62A4}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="20.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="31.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="31.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -736,7 +736,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -747,7 +747,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -758,7 +758,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>4</v>
       </c>
@@ -771,20 +771,21 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4969FD67-2E2F-4920-8A24-9B3F6A7CB976}">
   <dimension ref="A1:C8"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="8.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="41.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="8.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="41.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -795,7 +796,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>13</v>
       </c>
@@ -806,7 +807,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>13</v>
       </c>
@@ -817,7 +818,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>13</v>
       </c>
@@ -828,7 +829,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>13</v>
       </c>
@@ -839,7 +840,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>13</v>
       </c>
@@ -850,7 +851,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>13</v>
       </c>
@@ -861,7 +862,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>13</v>
       </c>
@@ -881,13 +882,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{08D4F942-EBC7-4392-9497-9CD173C449CD}">
   <dimension ref="A1:C30"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="21.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="106.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.88671875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="106.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -898,7 +899,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -909,7 +910,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -920,7 +921,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>4</v>
       </c>
@@ -931,7 +932,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>4</v>
       </c>
@@ -942,7 +943,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>4</v>
       </c>
@@ -953,7 +954,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>4</v>
       </c>
@@ -964,7 +965,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>4</v>
       </c>
@@ -975,7 +976,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>4</v>
       </c>
@@ -986,7 +987,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>4</v>
       </c>
@@ -997,7 +998,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>4</v>
       </c>
@@ -1008,7 +1009,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>4</v>
       </c>
@@ -1019,7 +1020,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>4</v>
       </c>
@@ -1030,7 +1031,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>4</v>
       </c>
@@ -1041,7 +1042,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>4</v>
       </c>
@@ -1052,7 +1053,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>4</v>
       </c>
@@ -1063,7 +1064,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>4</v>
       </c>
@@ -1074,7 +1075,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>4</v>
       </c>
@@ -1085,7 +1086,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>4</v>
       </c>
@@ -1096,7 +1097,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>4</v>
       </c>
@@ -1107,7 +1108,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>4</v>
       </c>
@@ -1118,7 +1119,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>4</v>
       </c>
@@ -1129,7 +1130,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>4</v>
       </c>
@@ -1140,7 +1141,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>4</v>
       </c>
@@ -1151,7 +1152,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>4</v>
       </c>
@@ -1162,7 +1163,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>4</v>
       </c>
@@ -1173,7 +1174,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>4</v>
       </c>
@@ -1184,7 +1185,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>4</v>
       </c>
@@ -1195,7 +1196,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>4</v>
       </c>
@@ -1206,7 +1207,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>4</v>
       </c>
@@ -1225,14 +1226,14 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1EEE61CD-3237-422A-82E8-CA9710108D17}">
   <dimension ref="A1:C10"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="16.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="91.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.88671875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="91.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1243,7 +1244,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -1254,7 +1255,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -1265,7 +1266,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>4</v>
       </c>
@@ -1276,7 +1277,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>4</v>
       </c>
@@ -1287,7 +1288,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>4</v>
       </c>
@@ -1298,7 +1299,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>4</v>
       </c>
@@ -1309,7 +1310,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>4</v>
       </c>
@@ -1320,7 +1321,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>4</v>
       </c>
@@ -1331,7 +1332,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>4</v>
       </c>
@@ -1351,12 +1352,12 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BFC7A54C-E16D-458B-92CE-DB4DE5E21708}">
   <dimension ref="A1:B8"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -1364,7 +1365,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -1372,7 +1373,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>7</v>
       </c>
@@ -1380,7 +1381,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>10</v>
       </c>
@@ -1388,22 +1389,22 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="B5" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="B6" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="B7" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="B8" t="s">
         <v>22</v>
       </c>
@@ -1416,14 +1417,14 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7B6B17DB-D82F-41EF-9E76-B6B556CE0B3E}">
   <dimension ref="A1:C5"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="16.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="19.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="20.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1434,7 +1435,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>84</v>
       </c>
@@ -1445,7 +1446,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>84</v>
       </c>
@@ -1456,7 +1457,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>84</v>
       </c>
@@ -1467,7 +1468,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>84</v>
       </c>

</xml_diff>

<commit_message>
Added and fixed TC
</commit_message>
<xml_diff>
--- a/src/main/resources/DeskReview_Field_Values.xlsx
+++ b/src/main/resources/DeskReview_Field_Values.xlsx
@@ -1,24 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="21727"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="22130"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\govgrants-product-automation\src\main\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Product Automation\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{027C3F22-D88C-4FD7-AD12-3CAD3626E955}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DEAB3C90-B34B-4EBE-A12B-2B368ECBA2D7}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{9AB3C168-78A6-4CA6-B0EE-C4F246080D71}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="3" xr2:uid="{9AB3C168-78A6-4CA6-B0EE-C4F246080D71}"/>
   </bookViews>
   <sheets>
     <sheet name="Creation" sheetId="1" r:id="rId1"/>
     <sheet name="Edition" sheetId="3" r:id="rId2"/>
-    <sheet name="Form Fields1" sheetId="5" r:id="rId3"/>
-    <sheet name="Form Fields" sheetId="7" r:id="rId4"/>
-    <sheet name="Sheet" sheetId="4" r:id="rId5"/>
-    <sheet name="Outcomes" sheetId="6" r:id="rId6"/>
+    <sheet name="SourceError" sheetId="8" r:id="rId3"/>
+    <sheet name="InstructionError" sheetId="9" r:id="rId4"/>
+    <sheet name="Form Fields1" sheetId="5" r:id="rId5"/>
+    <sheet name="Form Fields" sheetId="7" r:id="rId6"/>
+    <sheet name="Sheet" sheetId="4" r:id="rId7"/>
+    <sheet name="Outcomes" sheetId="6" r:id="rId8"/>
   </sheets>
   <calcPr calcId="179017"/>
   <extLst>
@@ -30,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="181" uniqueCount="108">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="219" uniqueCount="108">
   <si>
     <t>Sub Tab</t>
   </si>
@@ -719,13 +721,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27F20A35-8E6F-4015-873C-76781E4C62A4}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="20.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="31.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="31.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -736,7 +738,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -747,7 +749,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -758,7 +760,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>4</v>
       </c>
@@ -778,14 +780,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4969FD67-2E2F-4920-8A24-9B3F6A7CB976}">
   <dimension ref="A1:C8"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="8.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="41.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="41.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -796,7 +798,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>13</v>
       </c>
@@ -807,7 +809,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>13</v>
       </c>
@@ -818,7 +820,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>13</v>
       </c>
@@ -829,7 +831,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>13</v>
       </c>
@@ -840,7 +842,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>13</v>
       </c>
@@ -851,7 +853,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>13</v>
       </c>
@@ -862,7 +864,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>13</v>
       </c>
@@ -880,15 +882,15 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{08D4F942-EBC7-4392-9497-9CD173C449CD}">
-  <dimension ref="A1:C30"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2A26CCC8-9D00-4BF3-A8AD-20D2DBFACF71}">
+  <dimension ref="A1:C7"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="21.88671875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="106.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="38" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="46" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -899,323 +901,70 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="B2" t="s">
-        <v>23</v>
-      </c>
-      <c r="C2" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+        <v>15</v>
+      </c>
+      <c r="C2">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="B3" t="s">
-        <v>25</v>
-      </c>
-      <c r="C3" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+        <v>16</v>
+      </c>
+      <c r="C3">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>4</v>
-      </c>
-      <c r="B4" t="s">
-        <v>27</v>
+        <v>13</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>103</v>
       </c>
       <c r="C4" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>4</v>
-      </c>
-      <c r="B5" t="s">
-        <v>29</v>
+        <v>13</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>104</v>
       </c>
       <c r="C5" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>4</v>
-      </c>
-      <c r="B6" t="s">
-        <v>31</v>
+        <v>13</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>105</v>
       </c>
       <c r="C6" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>4</v>
-      </c>
-      <c r="B7" t="s">
-        <v>33</v>
+        <v>13</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>107</v>
       </c>
       <c r="C7" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>4</v>
-      </c>
-      <c r="B8" t="s">
-        <v>35</v>
-      </c>
-      <c r="C8" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>4</v>
-      </c>
-      <c r="B9" t="s">
-        <v>37</v>
-      </c>
-      <c r="C9" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
-        <v>4</v>
-      </c>
-      <c r="B10" t="s">
-        <v>39</v>
-      </c>
-      <c r="C10" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
-        <v>4</v>
-      </c>
-      <c r="B11" t="s">
-        <v>41</v>
-      </c>
-      <c r="C11" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
-        <v>4</v>
-      </c>
-      <c r="B12" t="s">
-        <v>43</v>
-      </c>
-      <c r="C12" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A13" t="s">
-        <v>4</v>
-      </c>
-      <c r="B13" t="s">
-        <v>45</v>
-      </c>
-      <c r="C13" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A14" t="s">
-        <v>4</v>
-      </c>
-      <c r="B14" t="s">
-        <v>47</v>
-      </c>
-      <c r="C14" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A15" t="s">
-        <v>4</v>
-      </c>
-      <c r="B15" t="s">
-        <v>49</v>
-      </c>
-      <c r="C15" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A16" t="s">
-        <v>4</v>
-      </c>
-      <c r="B16" t="s">
-        <v>51</v>
-      </c>
-      <c r="C16" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A17" t="s">
-        <v>4</v>
-      </c>
-      <c r="B17" t="s">
-        <v>53</v>
-      </c>
-      <c r="C17" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A18" t="s">
-        <v>4</v>
-      </c>
-      <c r="B18" t="s">
-        <v>55</v>
-      </c>
-      <c r="C18" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A19" t="s">
-        <v>4</v>
-      </c>
-      <c r="B19" t="s">
-        <v>57</v>
-      </c>
-      <c r="C19" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A20" t="s">
-        <v>4</v>
-      </c>
-      <c r="B20" t="s">
-        <v>59</v>
-      </c>
-      <c r="C20" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A21" t="s">
-        <v>4</v>
-      </c>
-      <c r="B21" t="s">
-        <v>61</v>
-      </c>
-      <c r="C21" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A22" t="s">
-        <v>4</v>
-      </c>
-      <c r="B22" t="s">
-        <v>63</v>
-      </c>
-      <c r="C22" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A23" t="s">
-        <v>4</v>
-      </c>
-      <c r="B23" t="s">
-        <v>65</v>
-      </c>
-      <c r="C23" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A24" t="s">
-        <v>4</v>
-      </c>
-      <c r="B24" t="s">
-        <v>67</v>
-      </c>
-      <c r="C24" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A25" t="s">
-        <v>4</v>
-      </c>
-      <c r="B25" t="s">
-        <v>69</v>
-      </c>
-      <c r="C25" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A26" t="s">
-        <v>4</v>
-      </c>
-      <c r="B26" t="s">
-        <v>71</v>
-      </c>
-      <c r="C26" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A27" t="s">
-        <v>4</v>
-      </c>
-      <c r="B27" t="s">
-        <v>73</v>
-      </c>
-      <c r="C27" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A28" t="s">
-        <v>4</v>
-      </c>
-      <c r="B28" t="s">
-        <v>75</v>
-      </c>
-      <c r="C28" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A29" t="s">
-        <v>4</v>
-      </c>
-      <c r="B29" t="s">
-        <v>77</v>
-      </c>
-      <c r="C29" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A30" t="s">
-        <v>4</v>
-      </c>
-      <c r="B30" t="s">
-        <v>79</v>
-      </c>
-      <c r="C30" t="s">
-        <v>62</v>
+        <v>18</v>
       </c>
     </row>
   </sheetData>
@@ -1224,16 +973,451 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BEDB83CE-C8E5-44AF-AE3C-DF3141462411}">
+  <dimension ref="A1:C7"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="38" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="41.85546875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C2">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C3">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>13</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="C4" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>13</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="C5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>13</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="C6" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>13</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="C7" t="s">
+        <v>18</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{08D4F942-EBC7-4392-9497-9CD173C449CD}">
+  <dimension ref="A1:C30"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="21.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="106.28515625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C2" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C3" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4" t="s">
+        <v>27</v>
+      </c>
+      <c r="C4" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>29</v>
+      </c>
+      <c r="C5" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>4</v>
+      </c>
+      <c r="B6" t="s">
+        <v>31</v>
+      </c>
+      <c r="C6" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>4</v>
+      </c>
+      <c r="B7" t="s">
+        <v>33</v>
+      </c>
+      <c r="C7" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>4</v>
+      </c>
+      <c r="B8" t="s">
+        <v>35</v>
+      </c>
+      <c r="C8" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>4</v>
+      </c>
+      <c r="B9" t="s">
+        <v>37</v>
+      </c>
+      <c r="C9" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>4</v>
+      </c>
+      <c r="B10" t="s">
+        <v>39</v>
+      </c>
+      <c r="C10" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>4</v>
+      </c>
+      <c r="B11" t="s">
+        <v>41</v>
+      </c>
+      <c r="C11" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>4</v>
+      </c>
+      <c r="B12" t="s">
+        <v>43</v>
+      </c>
+      <c r="C12" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>4</v>
+      </c>
+      <c r="B13" t="s">
+        <v>45</v>
+      </c>
+      <c r="C13" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>4</v>
+      </c>
+      <c r="B14" t="s">
+        <v>47</v>
+      </c>
+      <c r="C14" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>4</v>
+      </c>
+      <c r="B15" t="s">
+        <v>49</v>
+      </c>
+      <c r="C15" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>4</v>
+      </c>
+      <c r="B16" t="s">
+        <v>51</v>
+      </c>
+      <c r="C16" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>4</v>
+      </c>
+      <c r="B17" t="s">
+        <v>53</v>
+      </c>
+      <c r="C17" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>4</v>
+      </c>
+      <c r="B18" t="s">
+        <v>55</v>
+      </c>
+      <c r="C18" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>4</v>
+      </c>
+      <c r="B19" t="s">
+        <v>57</v>
+      </c>
+      <c r="C19" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>4</v>
+      </c>
+      <c r="B20" t="s">
+        <v>59</v>
+      </c>
+      <c r="C20" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>4</v>
+      </c>
+      <c r="B21" t="s">
+        <v>61</v>
+      </c>
+      <c r="C21" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>4</v>
+      </c>
+      <c r="B22" t="s">
+        <v>63</v>
+      </c>
+      <c r="C22" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>4</v>
+      </c>
+      <c r="B23" t="s">
+        <v>65</v>
+      </c>
+      <c r="C23" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>4</v>
+      </c>
+      <c r="B24" t="s">
+        <v>67</v>
+      </c>
+      <c r="C24" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>4</v>
+      </c>
+      <c r="B25" t="s">
+        <v>69</v>
+      </c>
+      <c r="C25" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>4</v>
+      </c>
+      <c r="B26" t="s">
+        <v>71</v>
+      </c>
+      <c r="C26" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>4</v>
+      </c>
+      <c r="B27" t="s">
+        <v>73</v>
+      </c>
+      <c r="C27" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>4</v>
+      </c>
+      <c r="B28" t="s">
+        <v>75</v>
+      </c>
+      <c r="C28" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>4</v>
+      </c>
+      <c r="B29" t="s">
+        <v>77</v>
+      </c>
+      <c r="C29" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>4</v>
+      </c>
+      <c r="B30" t="s">
+        <v>79</v>
+      </c>
+      <c r="C30" t="s">
+        <v>62</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1EEE61CD-3237-422A-82E8-CA9710108D17}">
   <dimension ref="A1:C10"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.88671875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="91.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="91.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1244,7 +1428,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -1255,7 +1439,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -1266,7 +1450,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>4</v>
       </c>
@@ -1277,7 +1461,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>4</v>
       </c>
@@ -1288,7 +1472,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>4</v>
       </c>
@@ -1299,7 +1483,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>4</v>
       </c>
@@ -1310,7 +1494,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>4</v>
       </c>
@@ -1321,7 +1505,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>4</v>
       </c>
@@ -1332,7 +1516,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>4</v>
       </c>
@@ -1349,15 +1533,15 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BFC7A54C-E16D-458B-92CE-DB4DE5E21708}">
   <dimension ref="A1:B8"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="9.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -1365,7 +1549,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -1373,7 +1557,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>7</v>
       </c>
@@ -1381,7 +1565,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>10</v>
       </c>
@@ -1389,22 +1573,22 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B7" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
         <v>22</v>
       </c>
@@ -1414,17 +1598,17 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7B6B17DB-D82F-41EF-9E76-B6B556CE0B3E}">
   <dimension ref="A1:C5"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="19.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="20.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1435,7 +1619,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>84</v>
       </c>
@@ -1446,7 +1630,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>84</v>
       </c>
@@ -1457,7 +1641,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>84</v>
       </c>
@@ -1468,7 +1652,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>84</v>
       </c>

</xml_diff>

<commit_message>
updated site visit and desk review feature files
</commit_message>
<xml_diff>
--- a/src/main/resources/DeskReview_Field_Values.xlsx
+++ b/src/main/resources/DeskReview_Field_Values.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="22430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="22730"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8954C04-E1AE-4D38-B8D6-D6F23A7D7A2D}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D141F2F6-3A58-4A38-B1BF-298166EF067C}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="7" xr2:uid="{9AB3C168-78A6-4CA6-B0EE-C4F246080D71}"/>
+    <workbookView xWindow="5304" yWindow="1500" windowWidth="17280" windowHeight="8964" xr2:uid="{9AB3C168-78A6-4CA6-B0EE-C4F246080D71}"/>
   </bookViews>
   <sheets>
     <sheet name="Creation" sheetId="1" r:id="rId1"/>
@@ -271,9 +271,6 @@
     <t>CheckListComment50__c</t>
   </si>
   <si>
-    <t>Automation Desk Review</t>
-  </si>
-  <si>
     <t>ActivityDescription__c</t>
   </si>
   <si>
@@ -356,6 +353,9 @@
   </si>
   <si>
     <t>Automation SPI</t>
+  </si>
+  <si>
+    <t>Automation Award Runtime Desk Review</t>
   </si>
 </sst>
 </file>
@@ -746,7 +746,7 @@
         <v>6</v>
       </c>
       <c r="C2" t="s">
-        <v>79</v>
+        <v>107</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
@@ -757,7 +757,7 @@
         <v>8</v>
       </c>
       <c r="C3" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
@@ -825,7 +825,7 @@
         <v>12</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C4" t="s">
         <v>17</v>
@@ -836,7 +836,7 @@
         <v>12</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C5" t="s">
         <v>17</v>
@@ -847,7 +847,7 @@
         <v>12</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C6" t="s">
         <v>19</v>
@@ -858,7 +858,7 @@
         <v>12</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C7" t="s">
         <v>20</v>
@@ -869,7 +869,7 @@
         <v>12</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C8" t="s">
         <v>17</v>
@@ -928,7 +928,7 @@
         <v>12</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C4" t="s">
         <v>17</v>
@@ -939,7 +939,7 @@
         <v>12</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C5" t="s">
         <v>17</v>
@@ -950,7 +950,7 @@
         <v>12</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C6" t="s">
         <v>19</v>
@@ -961,7 +961,7 @@
         <v>12</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C7" t="s">
         <v>17</v>
@@ -1019,7 +1019,7 @@
         <v>12</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C4" t="s">
         <v>17</v>
@@ -1030,7 +1030,7 @@
         <v>12</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C5" t="s">
         <v>19</v>
@@ -1041,7 +1041,7 @@
         <v>12</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C6" t="s">
         <v>20</v>
@@ -1052,7 +1052,7 @@
         <v>12</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C7" t="s">
         <v>17</v>
@@ -1436,7 +1436,7 @@
         <v>70</v>
       </c>
       <c r="C2" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
@@ -1447,7 +1447,7 @@
         <v>72</v>
       </c>
       <c r="C3" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
@@ -1458,7 +1458,7 @@
         <v>74</v>
       </c>
       <c r="C4" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
@@ -1469,7 +1469,7 @@
         <v>76</v>
       </c>
       <c r="C5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
@@ -1477,10 +1477,10 @@
         <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C6" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
@@ -1488,10 +1488,10 @@
         <v>4</v>
       </c>
       <c r="B7" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C7" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
@@ -1499,10 +1499,10 @@
         <v>4</v>
       </c>
       <c r="B8" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C8" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.3">
@@ -1510,10 +1510,10 @@
         <v>4</v>
       </c>
       <c r="B9" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C9" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.3">
@@ -1521,10 +1521,10 @@
         <v>4</v>
       </c>
       <c r="B10" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C10" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
   </sheetData>
@@ -1621,46 +1621,46 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>6</v>
       </c>
       <c r="C2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="C3" t="s">
         <v>83</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="C3" t="s">
-        <v>84</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C4" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C5" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated spreadsheet for desk review
</commit_message>
<xml_diff>
--- a/src/main/resources/DeskReview_Field_Values.xlsx
+++ b/src/main/resources/DeskReview_Field_Values.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\govgrants-product-automation\src\main\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MCPL#L92\Desktop\Automation projects\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{487BAD0D-C6E6-459A-B6A1-B1E73792FC18}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF815BD3-9809-47E1-82F7-D4AD3BE03AA6}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="7" xr2:uid="{9AB3C168-78A6-4CA6-B0EE-C4F246080D71}"/>
+    <workbookView xWindow="4097" yWindow="1029" windowWidth="16457" windowHeight="8554" activeTab="6" xr2:uid="{9AB3C168-78A6-4CA6-B0EE-C4F246080D71}"/>
   </bookViews>
   <sheets>
     <sheet name="Creation" sheetId="1" r:id="rId1"/>
@@ -355,7 +355,7 @@
     <t>Automation SPI</t>
   </si>
   <si>
-    <t>Automation Runtime Award Desk Review</t>
+    <t>Automation Runtime Award Desk</t>
   </si>
 </sst>
 </file>
@@ -731,13 +731,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27F20A35-8E6F-4015-873C-76781E4C62A4}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="2" max="2" width="20.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="31.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.53515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="31.07421875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -748,7 +748,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -759,7 +759,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -770,7 +770,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>4</v>
       </c>
@@ -790,14 +790,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4969FD67-2E2F-4920-8A24-9B3F6A7CB976}">
   <dimension ref="A1:C8"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="8.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="41.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="8.69140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.3046875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="41.3046875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -808,7 +808,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>12</v>
       </c>
@@ -819,7 +819,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>12</v>
       </c>
@@ -830,7 +830,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>12</v>
       </c>
@@ -841,7 +841,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>12</v>
       </c>
@@ -852,7 +852,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>12</v>
       </c>
@@ -863,7 +863,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>12</v>
       </c>
@@ -874,7 +874,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A8" t="s">
         <v>12</v>
       </c>
@@ -894,13 +894,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2A26CCC8-9D00-4BF3-A8AD-20D2DBFACF71}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="2" max="2" width="38" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="46" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -911,7 +911,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>12</v>
       </c>
@@ -922,7 +922,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>12</v>
       </c>
@@ -933,7 +933,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>12</v>
       </c>
@@ -944,7 +944,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>12</v>
       </c>
@@ -955,7 +955,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>12</v>
       </c>
@@ -966,7 +966,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>12</v>
       </c>
@@ -985,13 +985,13 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BEDB83CE-C8E5-44AF-AE3C-DF3141462411}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="2" max="2" width="38" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="41.88671875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="41.84375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1002,7 +1002,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>12</v>
       </c>
@@ -1013,7 +1013,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>12</v>
       </c>
@@ -1024,7 +1024,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>12</v>
       </c>
@@ -1035,7 +1035,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>12</v>
       </c>
@@ -1046,7 +1046,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>12</v>
       </c>
@@ -1057,7 +1057,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>12</v>
       </c>
@@ -1076,13 +1076,13 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{08D4F942-EBC7-4392-9497-9CD173C449CD}">
   <dimension ref="A1:C30"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="2" max="2" width="21.88671875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="106.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.84375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="106.3046875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1093,7 +1093,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -1104,7 +1104,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -1115,7 +1115,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>4</v>
       </c>
@@ -1126,7 +1126,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>4</v>
       </c>
@@ -1137,7 +1137,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>4</v>
       </c>
@@ -1148,7 +1148,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>4</v>
       </c>
@@ -1159,7 +1159,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A8" t="s">
         <v>4</v>
       </c>
@@ -1170,7 +1170,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A9" t="s">
         <v>4</v>
       </c>
@@ -1181,7 +1181,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A10" t="s">
         <v>4</v>
       </c>
@@ -1192,7 +1192,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A11" t="s">
         <v>4</v>
       </c>
@@ -1203,7 +1203,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A12" t="s">
         <v>4</v>
       </c>
@@ -1214,7 +1214,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A13" t="s">
         <v>4</v>
       </c>
@@ -1225,7 +1225,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A14" t="s">
         <v>4</v>
       </c>
@@ -1236,7 +1236,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A15" t="s">
         <v>4</v>
       </c>
@@ -1247,7 +1247,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A16" t="s">
         <v>4</v>
       </c>
@@ -1258,7 +1258,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A17" t="s">
         <v>4</v>
       </c>
@@ -1269,7 +1269,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A18" t="s">
         <v>4</v>
       </c>
@@ -1280,7 +1280,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A19" t="s">
         <v>4</v>
       </c>
@@ -1291,7 +1291,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A20" t="s">
         <v>4</v>
       </c>
@@ -1302,7 +1302,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A21" t="s">
         <v>4</v>
       </c>
@@ -1313,7 +1313,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A22" t="s">
         <v>4</v>
       </c>
@@ -1324,7 +1324,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A23" t="s">
         <v>4</v>
       </c>
@@ -1335,7 +1335,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A24" t="s">
         <v>4</v>
       </c>
@@ -1346,7 +1346,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A25" t="s">
         <v>4</v>
       </c>
@@ -1357,7 +1357,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A26" t="s">
         <v>4</v>
       </c>
@@ -1368,7 +1368,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A27" t="s">
         <v>4</v>
       </c>
@@ -1379,7 +1379,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A28" t="s">
         <v>4</v>
       </c>
@@ -1390,7 +1390,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A29" t="s">
         <v>4</v>
       </c>
@@ -1401,7 +1401,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A30" t="s">
         <v>4</v>
       </c>
@@ -1420,14 +1420,14 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1EEE61CD-3237-422A-82E8-CA9710108D17}">
   <dimension ref="A1:C10"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="16.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.88671875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="91.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.4609375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.84375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="91.3046875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1438,7 +1438,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -1449,7 +1449,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -1460,7 +1460,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>4</v>
       </c>
@@ -1471,7 +1471,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>4</v>
       </c>
@@ -1482,7 +1482,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>4</v>
       </c>
@@ -1493,7 +1493,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>4</v>
       </c>
@@ -1504,7 +1504,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A8" t="s">
         <v>4</v>
       </c>
@@ -1515,7 +1515,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A9" t="s">
         <v>4</v>
       </c>
@@ -1526,7 +1526,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A10" t="s">
         <v>4</v>
       </c>
@@ -1546,12 +1546,12 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BFC7A54C-E16D-458B-92CE-DB4DE5E21708}">
   <dimension ref="A1:B8"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="2" max="2" width="9.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.53515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -1559,7 +1559,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -1567,7 +1567,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>7</v>
       </c>
@@ -1575,7 +1575,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1583,22 +1583,22 @@
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.4">
       <c r="B5" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.4">
       <c r="B6" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.4">
       <c r="B7" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.4">
       <c r="B8" t="s">
         <v>21</v>
       </c>
@@ -1611,14 +1611,14 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7B6B17DB-D82F-41EF-9E76-B6B556CE0B3E}">
   <dimension ref="A1:C5"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="16.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="19.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="20.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.4609375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.3046875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.53515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1629,7 +1629,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" s="1" t="s">
         <v>82</v>
       </c>
@@ -1640,7 +1640,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" s="1" t="s">
         <v>82</v>
       </c>
@@ -1651,7 +1651,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" s="1" t="s">
         <v>82</v>
       </c>
@@ -1662,7 +1662,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A5" s="1" t="s">
         <v>82</v>
       </c>

</xml_diff>

<commit_message>
Refactored Closeout ,Progress Report, Site Visit, Application Intake, Auditor, Negotiation, Payment Request(partially)
</commit_message>
<xml_diff>
--- a/src/main/resources/DeskReview_Field_Values.xlsx
+++ b/src/main/resources/DeskReview_Field_Values.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Workpace-gov-grants-framework-automation\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A844DC25-9CB4-460A-8C9A-D4845104B533}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95A04784-6546-48D0-A55F-5738AA7CC24E}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-20610" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{9AB3C168-78A6-4CA6-B0EE-C4F246080D71}"/>
   </bookViews>
@@ -352,17 +352,17 @@
     <t>fieldSupportingCommentsQuestion1__c</t>
   </si>
   <si>
+    <t>Automation SPI3</t>
+  </si>
+  <si>
     <t>Automation Runtime Award Desk</t>
-  </si>
-  <si>
-    <t>Automation SPI3</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -380,7 +380,7 @@
       <b/>
       <sz val="9.8000000000000007"/>
       <color rgb="FF297BDE"/>
-      <name val="Consolas"/>
+      <name val="JetBrains Mono"/>
       <family val="3"/>
     </font>
   </fonts>
@@ -731,13 +731,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27F20A35-8E6F-4015-873C-76781E4C62A4}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="2" max="2" width="20.53125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="31.06640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="40.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -748,7 +748,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:3">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -756,10 +756,10 @@
         <v>6</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -767,10 +767,10 @@
         <v>8</v>
       </c>
       <c r="C3" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3">
       <c r="A4" t="s">
         <v>4</v>
       </c>
@@ -790,14 +790,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4969FD67-2E2F-4920-8A24-9B3F6A7CB976}">
   <dimension ref="A1:C8"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="8.6640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="30.33203125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="41.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -808,7 +808,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:3">
       <c r="A2" t="s">
         <v>12</v>
       </c>
@@ -819,7 +819,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:3">
       <c r="A3" t="s">
         <v>12</v>
       </c>
@@ -830,7 +830,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:3">
       <c r="A4" t="s">
         <v>12</v>
       </c>
@@ -841,7 +841,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:3">
       <c r="A5" t="s">
         <v>12</v>
       </c>
@@ -852,7 +852,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:3">
       <c r="A6" t="s">
         <v>12</v>
       </c>
@@ -863,7 +863,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:3">
       <c r="A7" t="s">
         <v>12</v>
       </c>
@@ -874,7 +874,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:3">
       <c r="A8" t="s">
         <v>12</v>
       </c>
@@ -894,13 +894,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2A26CCC8-9D00-4BF3-A8AD-20D2DBFACF71}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="2" max="2" width="38" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="46" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -911,7 +911,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:3">
       <c r="A2" t="s">
         <v>12</v>
       </c>
@@ -922,7 +922,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:3">
       <c r="A3" t="s">
         <v>12</v>
       </c>
@@ -933,7 +933,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:3">
       <c r="A4" t="s">
         <v>12</v>
       </c>
@@ -944,7 +944,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:3">
       <c r="A5" t="s">
         <v>12</v>
       </c>
@@ -955,7 +955,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:3">
       <c r="A6" t="s">
         <v>12</v>
       </c>
@@ -966,7 +966,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:3">
       <c r="A7" t="s">
         <v>12</v>
       </c>
@@ -985,13 +985,13 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BEDB83CE-C8E5-44AF-AE3C-DF3141462411}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="2" max="2" width="38" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="41.86328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1002,7 +1002,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:3">
       <c r="A2" t="s">
         <v>12</v>
       </c>
@@ -1013,7 +1013,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:3">
       <c r="A3" t="s">
         <v>12</v>
       </c>
@@ -1024,7 +1024,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:3">
       <c r="A4" t="s">
         <v>12</v>
       </c>
@@ -1035,7 +1035,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:3">
       <c r="A5" t="s">
         <v>12</v>
       </c>
@@ -1046,7 +1046,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:3">
       <c r="A6" t="s">
         <v>12</v>
       </c>
@@ -1057,7 +1057,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:3">
       <c r="A7" t="s">
         <v>12</v>
       </c>
@@ -1076,13 +1076,13 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{08D4F942-EBC7-4392-9497-9CD173C449CD}">
   <dimension ref="A1:C30"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="2" max="2" width="21.86328125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="106.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1093,7 +1093,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:3">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -1104,7 +1104,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:3">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -1115,7 +1115,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:3">
       <c r="A4" t="s">
         <v>4</v>
       </c>
@@ -1126,7 +1126,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:3">
       <c r="A5" t="s">
         <v>4</v>
       </c>
@@ -1137,7 +1137,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:3">
       <c r="A6" t="s">
         <v>4</v>
       </c>
@@ -1148,7 +1148,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:3">
       <c r="A7" t="s">
         <v>4</v>
       </c>
@@ -1159,7 +1159,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:3">
       <c r="A8" t="s">
         <v>4</v>
       </c>
@@ -1170,7 +1170,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:3">
       <c r="A9" t="s">
         <v>4</v>
       </c>
@@ -1181,7 +1181,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:3">
       <c r="A10" t="s">
         <v>4</v>
       </c>
@@ -1192,7 +1192,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:3">
       <c r="A11" t="s">
         <v>4</v>
       </c>
@@ -1203,7 +1203,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:3">
       <c r="A12" t="s">
         <v>4</v>
       </c>
@@ -1214,7 +1214,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:3">
       <c r="A13" t="s">
         <v>4</v>
       </c>
@@ -1225,7 +1225,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:3">
       <c r="A14" t="s">
         <v>4</v>
       </c>
@@ -1236,7 +1236,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:3">
       <c r="A15" t="s">
         <v>4</v>
       </c>
@@ -1247,7 +1247,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:3">
       <c r="A16" t="s">
         <v>4</v>
       </c>
@@ -1258,7 +1258,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:3">
       <c r="A17" t="s">
         <v>4</v>
       </c>
@@ -1269,7 +1269,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:3">
       <c r="A18" t="s">
         <v>4</v>
       </c>
@@ -1280,7 +1280,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:3">
       <c r="A19" t="s">
         <v>4</v>
       </c>
@@ -1291,7 +1291,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:3">
       <c r="A20" t="s">
         <v>4</v>
       </c>
@@ -1302,7 +1302,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:3">
       <c r="A21" t="s">
         <v>4</v>
       </c>
@@ -1313,7 +1313,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:3">
       <c r="A22" t="s">
         <v>4</v>
       </c>
@@ -1324,7 +1324,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:3">
       <c r="A23" t="s">
         <v>4</v>
       </c>
@@ -1335,7 +1335,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:3">
       <c r="A24" t="s">
         <v>4</v>
       </c>
@@ -1346,7 +1346,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:3">
       <c r="A25" t="s">
         <v>4</v>
       </c>
@@ -1357,7 +1357,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:3">
       <c r="A26" t="s">
         <v>4</v>
       </c>
@@ -1368,7 +1368,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:3">
       <c r="A27" t="s">
         <v>4</v>
       </c>
@@ -1379,7 +1379,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="28" spans="1:3">
       <c r="A28" t="s">
         <v>4</v>
       </c>
@@ -1390,7 +1390,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="29" spans="1:3">
       <c r="A29" t="s">
         <v>4</v>
       </c>
@@ -1401,7 +1401,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="30" spans="1:3">
       <c r="A30" t="s">
         <v>4</v>
       </c>
@@ -1420,14 +1420,14 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1EEE61CD-3237-422A-82E8-CA9710108D17}">
   <dimension ref="A1:C10"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="16.46484375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="14.86328125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="91.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1438,7 +1438,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:3">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -1449,7 +1449,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:3">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -1460,7 +1460,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:3">
       <c r="A4" t="s">
         <v>4</v>
       </c>
@@ -1471,7 +1471,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:3">
       <c r="A5" t="s">
         <v>4</v>
       </c>
@@ -1482,7 +1482,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:3">
       <c r="A6" t="s">
         <v>4</v>
       </c>
@@ -1493,7 +1493,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:3">
       <c r="A7" t="s">
         <v>4</v>
       </c>
@@ -1504,7 +1504,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:3">
       <c r="A8" t="s">
         <v>4</v>
       </c>
@@ -1515,7 +1515,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:3">
       <c r="A9" t="s">
         <v>4</v>
       </c>
@@ -1526,7 +1526,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:3">
       <c r="A10" t="s">
         <v>4</v>
       </c>
@@ -1546,12 +1546,12 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BFC7A54C-E16D-458B-92CE-DB4DE5E21708}">
   <dimension ref="A1:B8"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="2" max="2" width="9.53125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:2">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -1559,7 +1559,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:2">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -1567,7 +1567,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:2">
       <c r="A3" t="s">
         <v>7</v>
       </c>
@@ -1575,7 +1575,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:2">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1583,22 +1583,22 @@
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:2">
       <c r="B5" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:2">
       <c r="B6" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:2">
       <c r="B7" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:2">
       <c r="B8" t="s">
         <v>21</v>
       </c>
@@ -1611,14 +1611,14 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7B6B17DB-D82F-41EF-9E76-B6B556CE0B3E}">
   <dimension ref="A1:C5"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="16.46484375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="19.33203125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="20.53125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1629,7 +1629,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:3">
       <c r="A2" s="1" t="s">
         <v>82</v>
       </c>
@@ -1640,7 +1640,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:3">
       <c r="A3" s="1" t="s">
         <v>82</v>
       </c>
@@ -1651,7 +1651,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:3">
       <c r="A4" s="1" t="s">
         <v>82</v>
       </c>
@@ -1662,7 +1662,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:3">
       <c r="A5" s="1" t="s">
         <v>82</v>
       </c>

</xml_diff>